<commit_message>
Changelog automatizado: Registro de cambio por GeanluisGL
</commit_message>
<xml_diff>
--- a/historial_cambios.xlsx
+++ b/historial_cambios.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,38 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>3930fd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:13:26</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GeanluisGL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Add files via upload</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>a9cf6ff</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: changelog automatizado [GeanluisGL]
</commit_message>
<xml_diff>
--- a/historial_cambios.xlsx
+++ b/historial_cambios.xlsx
@@ -17,8 +17,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -52,10 +52,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -561,8 +562,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46283.68477786391</v>
+      <c r="A5" s="3" t="n">
+        <v>46283.6847778588</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -588,6 +589,37 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>0ac331d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>46283.69043757788</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GeanluisGL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>master</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Add script to log changes in Excel file
+This script logs changes to an Excel file, capturing details such as user, branch, release, commit message, and commit ID.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>3c6c8b0</t>
         </is>
       </c>
     </row>

</xml_diff>